<commit_message>
análises circulares para publicação
</commit_message>
<xml_diff>
--- a/dados/tabela_polinizacao_final.xlsx
+++ b/dados/tabela_polinizacao_final.xlsx
@@ -1,113 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ecf526ac8f48663/Documentos/fenologia/dados/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_4E72FDCE8F79A8D366075C52F3D25A36CC03E7AA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{226CB515-C1C3-4510-955E-4FDF6DF7E6EE}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="-120" windowWidth="20640" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
-  <si>
-    <t>Sindrome</t>
-  </si>
-  <si>
-    <t>Melhor_Modelo</t>
-  </si>
-  <si>
-    <t>Distribuicao</t>
-  </si>
-  <si>
-    <t>n</t>
-  </si>
-  <si>
-    <t>Teste_Escolha</t>
-  </si>
-  <si>
-    <t>Estatistica</t>
-  </si>
-  <si>
-    <t>P_Valor</t>
-  </si>
-  <si>
-    <t>r_vetor</t>
-  </si>
-  <si>
-    <t>Angulo_Med_Rad</t>
-  </si>
-  <si>
-    <t>Data_Media</t>
-  </si>
-  <si>
-    <t>q1_rad</t>
-  </si>
-  <si>
-    <t>k1_kappa</t>
-  </si>
-  <si>
-    <t>q2_rad</t>
-  </si>
-  <si>
-    <t>k2_kappa</t>
-  </si>
-  <si>
-    <t>lambda</t>
-  </si>
-  <si>
-    <t>AICc</t>
-  </si>
-  <si>
-    <t>Peso_AIC</t>
-  </si>
-  <si>
-    <t>Zoofilia</t>
-  </si>
-  <si>
-    <t>M5A</t>
-  </si>
-  <si>
-    <t>Bimodal</t>
-  </si>
-  <si>
-    <t>Rao Spacing</t>
-  </si>
-  <si>
-    <t>20/09/22</t>
-  </si>
-  <si>
-    <t>Anemofilia</t>
-  </si>
-  <si>
-    <t>M2B</t>
-  </si>
-  <si>
-    <t>Unimodal</t>
-  </si>
-  <si>
-    <t>Rayleigh</t>
-  </si>
-  <si>
-    <t>11/10/22</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,21 +63,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -207,7 +107,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -241,7 +141,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -276,10 +175,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -452,173 +350,209 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sindrome</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Melhor_Modelo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distribuicao</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Teste_Escolha</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Estatistica</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>P_Valor</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>r_vetor</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Angulo_Med_Rad</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Data_Media</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>q1_rad</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>k1_kappa</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>q2_rad</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>k2_kappa</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>lambda</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>AICc</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Peso_AIC</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Zoofilia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>M5A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Bimodal</t>
+        </is>
       </c>
       <c r="D2">
         <v>133</v>
       </c>
-      <c r="E2" t="s">
-        <v>20</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Rao Spacing</t>
+        </is>
       </c>
       <c r="F2">
-        <v>330.22556390977451</v>
+        <v>330.2255639097745</v>
       </c>
       <c r="H2">
-        <v>0.42599999999999999</v>
+        <v>0.426</v>
       </c>
       <c r="I2">
-        <v>4.5259999999999998</v>
-      </c>
-      <c r="J2" t="s">
-        <v>21</v>
+        <v>4.526</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>20/09/22</t>
+        </is>
       </c>
       <c r="K2">
-        <v>4.2560000000000002</v>
+        <v>4.256</v>
       </c>
       <c r="L2">
-        <v>2.0190000000000001</v>
+        <v>2.019</v>
       </c>
       <c r="M2">
-        <v>0.39300000000000002</v>
+        <v>0.393</v>
       </c>
       <c r="N2">
-        <v>2.0190000000000001</v>
+        <v>2.019</v>
       </c>
       <c r="O2">
         <v>0.749</v>
       </c>
       <c r="P2">
-        <v>436.91500000000002</v>
+        <v>436.915</v>
       </c>
       <c r="Q2">
-        <v>0.68400000000000005</v>
+        <v>0.6840000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>24</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Anemofilia</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>M2B</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Unimodal</t>
+        </is>
       </c>
       <c r="D3">
         <v>6</v>
       </c>
-      <c r="E3" t="s">
-        <v>25</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Rayleigh</t>
+        </is>
       </c>
       <c r="F3">
-        <v>0.60872694941883998</v>
+        <v>0.60872694941884</v>
       </c>
       <c r="G3">
         <v>0.1058438991612469</v>
       </c>
       <c r="H3">
-        <v>0.60899999999999999</v>
+        <v>0.609</v>
       </c>
       <c r="I3">
-        <v>4.8739999999999997</v>
-      </c>
-      <c r="J3" t="s">
-        <v>26</v>
+        <v>4.874</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>11/10/22</t>
+        </is>
       </c>
       <c r="K3">
-        <v>4.9740000000000002</v>
+        <v>4.974</v>
       </c>
       <c r="L3">
         <v>226.999</v>
       </c>
       <c r="P3">
-        <v>9.1159999999999997</v>
+        <v>9.116</v>
       </c>
       <c r="Q3">
-        <v>0.66800000000000004</v>
+        <v>0.668</v>
       </c>
     </row>
   </sheetData>

</xml_diff>